<commit_message>
docs: close traceability gaps between v1.1 spec and MVP docs (3rd-round audit)
Converts 23 "diagnosed-only"/"missing" findings from the traceability audit
into actual buildable requirements: automation consent flow, skip buttons on
4 journey screens, recommendation scoring formula + response-time metric
source, external link-outs (issue/PR pages), Journey overview settings
toggle, and real GitHub/IDE integration in place of simulated actions.
Updates the requirements xlsx, screen-spec xlsx, IA, and ERD together so the
four stay consistent.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/그린커밋_화면정의서_MVP.xlsx
+++ b/docs/그린커밋_화면정의서_MVP.xlsx
@@ -608,7 +608,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>[정정 2026-07-20] fable 기반 논리 결함 재평가에서 21건을 발견해 요구사항정의서·화면정의서·IA 3개 문서에 반영했다. 화면정의서에서는 SCR000(전역 셸/TopBar)이 초판에서 통째로 누락돼 있던 것을 발견해 새로 추가했고, 기존 17개 화면 중 다수 요소에 [코드-스펙 괴리] 주석을 보강했다. 상세 근거는 요구사항정의서 표지 탭과 동일한 표기 규칙을 따른다.</t>
+          <t>[정정 2026-07-20] fable 기반 논리 결함 재평가에서 21건을 발견해 요구사항정의서·화면정의서·IA 3개 문서에 반영했다. 화면정의서에서는 SCR000(전역 셸/TopBar)이 초판에서 통째로 누락돼 있던 것을 발견해 새로 추가했고, 기존 17개 화면 중 다수 요소에 [코드-스펙 괴리] 주석을 보강했다. 상세 근거는 요구사항정의서 표지 탭과 동일한 표기 규칙을 따른다. 같은 날 이어진 3차(traceability) 재평가에서는 기획서 원문이 요구하지만 이전 판엔 진단만 있던 항목(자동화 동의 모달, 4개 화면 스킵 버튼, 원문 링크, IDE 6종, 검증 질문 확인, 실제 GitHub/IDE 연동 등)을 신규 요소로 추가했다([정정 2026-07-20, 요구사항으로 승격] 표기로 구분).</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>"이 권한을 받아요" 3항목(공개저장소·활동읽기 / Fork생성·PR열기자동화 / 비공개저장소·이메일 제외)</t>
+          <t>"이 권한을 받아요" 3항목(공개저장소·활동읽기 / Fork생성 자동화 / 비공개저장소·이메일 제외)</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] 이전 판은 존재하지 않는 'PR열기 자동화' 권한을 안내했음(PR 등록은 REQ-027에서 사용자가 URL을 직접 붙여넣는 완전 수동 방식) — 삭제</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>note: 권한 해제 안내 + BR06 언급</t>
+          <t>note: "권한은 언제든 설정에서 해제 가능, 자동화는 Fork 실행 시 별도 동의 모달에서 최종 확인 후 실행" — 실제 동의 확인 시점은 이 화면이 아니라 SCR009(REQ-015) 첫 자동화 클릭 시</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>BR06</t>
+          <t>BR05, BR06</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>BR01. [코드-스펙 괴리] 위 체크리스트가 안내하는 'Fork생성·PR열기 자동화' 권한(FORK_AUTOMATION/PR_AUTOMATION Consent)은 이 로그인 흐름에서 생성되지 않는다(PROFILE_READ/PUBLIC_REPO_READ 2건만 자동 생성) — 존재하지 않는 동의를 안내한 셈. PR열기 자동화 기능 자체도 MVP엔 없음(SCR012는 완전 수동 URL 등록)</t>
+          <t>BR01</t>
         </is>
       </c>
     </row>
@@ -1924,12 +1924,12 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(3, 단일선택)</t>
+          <t>버튼그룹(6, 단일선택)</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>주 IDE: VS Code / IntelliJ·JetBrains / 기타</t>
+          <t>주 IDE: VS Code / IntelliJ IDEA / PyCharm / WebStorm / Eclipse / 기타</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>enum 전체는 6종(PYCHARM/WEBSTORM/ECLIPSE 포함)이나 화면엔 3개만 노출</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] 이전 판은 enum 6종(PYCHARM/WEBSTORM/ECLIPSE 포함) 중 3개만 노출했음 — 전체 노출로 승격</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(3, 단일선택)</t>
+          <t>칩 편집 UI</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>외부 PR 경험: 0회 / 1~2회 / 3회+</t>
+          <t>"분석된 기술 스택 확인·보정" — SCR003 analyzedLanguages를 칩으로 표시, 클릭으로 추가/제거 가능</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>선택값 로컬state 저장</t>
+          <t>편집 결과를 userAdjustedSkills로 저장(BR02 자기진단 분리 표시 요건)</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] 이전 판은 이 편집 UI 자체가 없어 userAdjustedSkills가 완전 write-only 필드였음 — UI 신설</t>
         </is>
       </c>
     </row>
@@ -2023,12 +2023,12 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Git·PR 자신감: 없음 / 보통 / 능숙</t>
+          <t>외부 PR 경험: 0회 / 1~2회 / 3회+</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -2065,12 +2065,12 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(6, 다중선택)</t>
+          <t>버튼그룹(3, 단일선택)</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>관심분야: 공익/문서/웹/데이터/테스트/버그</t>
+          <t>Git·PR 자신감: 없음 / 보통 / 능숙</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>토글 방식 다중 선택</t>
+          <t>선택값 로컬state 저장</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(4, 단일선택)</t>
+          <t>버튼그룹(6, 다중선택)</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>주당 투자 가능 시간: 1시간미만/2~3시간/4~6시간/7시간+</t>
+          <t>관심분야: 공익/문서/웹/데이터/테스트/버그</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>선택값 로컬state 저장</t>
+          <t>토글 방식 다중 선택</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -2159,22 +2159,22 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(2, 단일선택)</t>
+          <t>버튼그룹(4, 단일선택)</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>첫 기여 여부: 네,처음이에요 / 아니요,해봤어요</t>
+          <t>주당 투자 가능 시간: 1시간미만/2~3시간/4~6시간/7시간+</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>필수(미선택 시 제출 차단)</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>초기값 null, BR03 분기 기준값</t>
+          <t>선택값 로컬state 저장</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>BR03</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2206,22 +2206,22 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>텍스트(조건부)</t>
+          <t>버튼그룹(2, 단일선택)</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>에러: '오픈소스 기여가 처음인지 알려주세요.'</t>
+          <t>첫 기여 여부: 네,처음이에요 / 아니요,해봤어요</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수(미선택 시 제출 차단)</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>isFirstTime===null 상태로 제출 시도 시</t>
+          <t>초기값 null, BR03 분기 기준값</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR03</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>에러: '저장에 실패했어요. 다시 시도해주세요.'</t>
+          <t>에러: '오픈소스 기여가 처음인지 알려주세요.'</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>API 실패 시</t>
+          <t>isFirstTime===null 상태로 제출 시도 시</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -2300,59 +2300,59 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>텍스트(조건부)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>"추천 받기 →" / "저장 중…"</t>
+          <t>에러: '저장에 실패했어요. 다시 시도해주세요.'</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>disabled=saving, 성공 시 isFirstTime===true → /onboarding/tutorial(SCR005), false → /recommend/repositories(SCR006)</t>
+          <t>API 실패 시</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>PUT /users/me/onboarding</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>BR03</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>SCR005</t>
+          <t>SCR004</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>초보자 튜토리얼</t>
+          <t>추가 프로필</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>SCR005-1</t>
+          <t>SCR004-10</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>h1 "오픈소스가 뭐예요? 🌍"</t>
+          <t>"추천 받기 →" / "저장 중…"</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -2362,17 +2362,17 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>disabled=saving, 성공 시 isFirstTime===true → /onboarding/tutorial(SCR005), false → /recommend/repositories(SCR006)</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PUT /users/me/onboarding</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR03</t>
         </is>
       </c>
     </row>
@@ -2389,17 +2389,17 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>SCR005-2</t>
+          <t>SCR005-1</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>"What" 블록 — 오픈소스 개념 설명</t>
+          <t>h1 "오픈소스가 뭐예요? 🌍"</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>SCR005-3</t>
+          <t>SCR005-2</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -2446,12 +2446,12 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>"이런 것도 다 기여예요" 3항목(오타수정/번역/예제추가)</t>
+          <t>"What" 블록 — 오픈소스 개념 설명</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2483,27 +2483,27 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>SCR005-4</t>
+          <t>SCR005-3</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>흐름도</t>
+          <t>카드</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Fork→고치기→PR→리뷰→Merge 5단계</t>
+          <t>"이런 것도 다 기여예요" 3항목(오타수정/번역/예제추가)</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>정적 다이어그램</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -2530,17 +2530,17 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>SCR005-5</t>
+          <t>SCR005-4</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>흐름도</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>"건너뛰기"</t>
+          <t>Fork→고치기→PR→리뷰→Merge 5단계</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -2550,12 +2550,12 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>disabled=saving, finish(true) → completed=false,skipped=true</t>
+          <t>정적 다이어그램</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>POST /tutorial/progress</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>SCR005-6</t>
+          <t>SCR005-5</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>"좋아, 시작해볼래 →"</t>
+          <t>"건너뛰기"</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>disabled=saving, finish(false) → completed=true,skipped=false. 둘 다 이후 /recommend/repositories(SCR006)로 이동</t>
+          <t>클릭 시 사유 선택 모달 노출 후 disabled=saving, finish(true, skipReason) → completed=false,skipped=true</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
@@ -2607,44 +2607,44 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>[코드-스펙 괴리][정정 2026-07-20] 이 화면은 Journey 세션 생성(SCR007) 이전에 지나가므로 JourneyStepType.TUTORIAL을 갱신할 세션이 애초에 없다 — 'TUTORIAL 완료 처리를 여기서 하면 된다'는 이전 제안은 시간순서상 성립하지 않는다. 근본 원인은 TUTORIAL이 Journey 9단계 안에 있는 설계 자체(요구사항정의서 REQ-009/상태전이 탭 참고) — TutorialProgress(이 화면이 실제로 쓰는 테이블)로 진행상태를 충분히 추적할 수 있다</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>SCR006</t>
+          <t>SCR005</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Repository 추천</t>
+          <t>초보자 튜토리얼</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>SCR006-1</t>
+          <t>SCR005-6</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>모달(조건부)</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>h1 "미션 찾기 — 레포부터 골라요"</t>
+          <t>사유 선택 1탭 — "이미 알아요" / "나중에 볼게요" / "그냥 넘어갈래요"(미선택도 스킵 자체는 허용)</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>위 '건너뛰기' 클릭 시</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -2654,24 +2654,24 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] UC02 완전누락(스킵 사유 미수집)을 신설(요구사항정의서 REQ-009 참고)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>SCR006</t>
+          <t>SCR005</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Repository 추천</t>
+          <t>초보자 튜토리얼</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>SCR006-2</t>
+          <t>SCR005-7</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2681,27 +2681,27 @@
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>"🔄 새로고침"</t>
+          <t>"좋아, 시작해볼래 →"</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>목록 재조회</t>
+          <t>disabled=saving, finish(false) → completed=true,skipped=false. 둘 다 이후 /recommend/repositories(SCR006)로 이동</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>GET /recommendations/repositories</t>
+          <t>POST /tutorial/progress</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[코드-스펙 괴리][정정 2026-07-20] 이 화면은 Journey 세션 생성(SCR007) 이전에 지나가므로 JourneyStepType.TUTORIAL을 갱신할 세션이 애초에 없다 — 'TUTORIAL 완료 처리를 여기서 하면 된다'는 이전 제안은 시간순서상 성립하지 않는다. 근본 원인은 TUTORIAL이 Journey 9단계 안에 있는 설계 자체(요구사항정의서 REQ-009/상태전이 탭 참고) — TutorialProgress(이 화면이 실제로 쓰는 테이블)로 진행상태를 충분히 추적할 수 있다</t>
         </is>
       </c>
     </row>
@@ -2718,17 +2718,17 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>SCR006-3</t>
+          <t>SCR006-1</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>카드목록(반복)</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>레포명 · 적합도pill · 설명 · 언어/stars태그 · 공익목적·최근활동·기여문서·응답성 표 · 빠른응답 배지(avgFeedbackHours≤48h) · 주의점 · evidence[0]</t>
+          <t>h1 "미션 찾기 — 레포부터 골라요"</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
@@ -2738,17 +2738,17 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>목록 렌더링</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>GET /recommendations/repositories</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>avgFeedbackHours는 수동 시드값 — BR09 표기 보강 권장. [코드-스펙 괴리][중대] '적합도'가 실제로는 개인화되지 않는다 — 이 API 호출에 userId가 안 실려서 SCR004에서 고른 관심분야가 전혀 반영되지 않는다(요구사항정의서 REQ-010 참고). 또한 이 GET은 호출마다 DB에 추천 데이터를 새로 저장하는 부작용이 있어(조회 API인데 쓰기 발생), 새로고침 버튼을 누를 때마다 고아 데이터가 쌓인다</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2765,32 +2765,32 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>SCR006-4</t>
+          <t>SCR006-2</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>버튼(카드 내 반복)</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>"이 레포 선택 →"</t>
+          <t>"🔄 새로고침"</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>/recommend/issues?repositoryId&amp;repositoryName (SCR007)로 이동</t>
+          <t>목록 재조회</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /recommendations/repositories</t>
         </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
@@ -2812,64 +2812,64 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>SCR006-5</t>
+          <t>SCR006-3</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>상태분기</t>
+          <t>카드목록(반복)</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>로딩중 / 에러</t>
+          <t>레포명 · 적합도pill(fitScore+관심분야 가산점+응답시간 가산점 산식, 요구사항정의서 REQ-010 참고) · 설명 · 언어/stars태그 · 공익목적·최근활동·기여문서·응답성 표 · "⚡ 메인테이너 첫 반응 예상 · 약 N시간" 배지(avgFeedbackHours 존재 시, "예상/약" 표현 필수 — BR09) · 주의점 · evidence[0]</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>"불러오는 중…" / "불러오지 못했어요. 새로고침해보세요."</t>
+          <t>목록 렌더링(userId 필수 전달)</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /recommendations/repositories</t>
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>avgFeedbackHours는 수동 시드값, maintainerResponseMetricSource로 산정 출처 표기(BR09). [정정 2026-07-20, 요구사항으로 승격] 이전 판 배지 문구 '⚡빠른응답·평균N시간'은 BR09가 금지하는 확정형 표현이라 삭제 — 위 '예상·약' 문구로 교체. userId 미전달로 개인화가 안 되는 것도 요구사항정의서 REQ-010에서 필수 전달로 승격. 이 GET은 호출마다 DB에 추천 데이터를 새로 저장하는 부작용이 있어(조회 API인데 쓰기 발생), 새로고침 버튼을 누를 때마다 고아 데이터가 쌓인다</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>SCR007</t>
+          <t>SCR006</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Issue 선택</t>
+          <t>Repository 추천</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>SCR007-1</t>
+          <t>SCR006-4</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>버튼(카드 내 반복)</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>h1 "미션 찾기 — 이슈 선택"</t>
+          <t>"이 레포 선택 →"</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>/recommend/issues?repositoryId&amp;repositoryName (SCR007)로 이동</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
@@ -2896,17 +2896,17 @@
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>SCR007</t>
+          <t>SCR006</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Issue 선택</t>
+          <t>Repository 추천</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>SCR007-2</t>
+          <t>SCR006-5</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>repositoryId 없음 / 에러 / 로딩중</t>
+          <t>로딩중 / 에러</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>"먼저 레포를 선택해주세요." 등</t>
+          <t>"불러오는 중…" / "불러오지 못했어요. 새로고침해보세요."</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>BR04</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>SCR007-3</t>
+          <t>SCR007-1</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>카드목록(반복)</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>제목·#번호 · 기여유형 태그 · 난이도 pill · 예상범위 pill · 현재문제 · 완료기준</t>
+          <t>h1 "미션 찾기 — 이슈 선택"</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
@@ -2973,12 +2973,12 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>목록 렌더링</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>GET /repositories/{id}/issues</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I50" s="7" t="inlineStr">
@@ -3000,27 +3000,27 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>SCR007-4</t>
+          <t>SCR007-2</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>버튼(카드 내 반복)</t>
+          <t>상태분기</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>"이 이슈 선택"</t>
+          <t>repositoryId 없음 / 에러 / 로딩중</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>setSelectedIssueId, 선택된 카드는 하이라이트</t>
+          <t>"먼저 레포를 선택해주세요." 등</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR04</t>
         </is>
       </c>
     </row>
@@ -3047,17 +3047,17 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>SCR007-5</t>
+          <t>SCR007-3</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>하단 고정바</t>
+          <t>카드목록(반복)</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>선택 레포·이슈 요약 텍스트</t>
+          <t>제목·#번호 · 기여유형 태그 · 난이도 pill · 예상범위 pill · 현재문제 · 완료기준 · "이슈 원문 보기 ↗" 링크(issue.url, 새 탭)</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -3067,17 +3067,17 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>실시간 반영</t>
+          <t>목록 렌더링</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /repositories/{id}/issues</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격, 권장사항] SCR010과 동일 링크를 여기서도 미리 제공(부록B '원문 링크 항상 제공' 권장 범위)</t>
         </is>
       </c>
     </row>
@@ -3094,17 +3094,17 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>SCR007-6</t>
+          <t>SCR007-4</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>버튼(카드 내 반복)</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>"다음 단계로(기여 시작) →" / "시작하는 중…"</t>
+          <t>"이 이슈 선택"</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>disabled=미선택 또는 진행중, 성공 시 /journey/overview(SCR008)로 이동</t>
+          <t>setSelectedIssueId, 선택된 카드는 하이라이트</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>POST /journeys</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I53" s="7" t="inlineStr">
@@ -3131,27 +3131,27 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>SCR008</t>
+          <t>SCR007</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Journey 개요</t>
+          <t>Issue 선택</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>SCR008-1</t>
+          <t>SCR007-5</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>하단 고정바</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>h1 "기여 여정 개요"</t>
+          <t>선택 레포·이슈 요약 텍스트</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>실시간 반영</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -3178,27 +3178,27 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>SCR008</t>
+          <t>SCR007</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Journey 개요</t>
+          <t>Issue 선택</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>SCR008-2</t>
+          <t>SCR007-6</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>"이번 Journey 진행상태" — 9단계 순서·상태 pill</t>
+          <t>"다음 단계로(기여 시작) →" / "시작하는 중…"</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -3208,17 +3208,17 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>실데이터 렌더링</t>
+          <t>disabled=미선택 또는 진행중, 성공 시 /journey/overview(SCR008)로 이동</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>GET /journeys/{id}</t>
+          <t>POST /journeys</t>
         </is>
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>[코드-스펙 괴리] 이 API 응답엔 레포·이슈 정보(meta)가 없어, 새로고침 시 이 카드 자체는 복구되지만 이후 화면(SCR009~013)은 meta 없이는 정상 동작하지 않는다 — '새로고침 복구용'이라는 이름이 이 카드에만 해당됨</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -3235,27 +3235,27 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>SCR008-3</t>
+          <t>SCR008-1</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>"단계별 스킵·자동화 Matrix" — 부록B 정적 표</t>
+          <t>h1 "기여 여정 개요"</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>정적 표시(보기 전용)</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
@@ -3265,7 +3265,7 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>[v1.1 설계target] 표19 원문은 설정 변경 UI도 요구하나 현재 보기전용</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -3282,17 +3282,17 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>SCR008-4</t>
+          <t>SCR008-2</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>버튼(Link)</t>
+          <t>카드</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>"Fork부터 시작할게요 →"</t>
+          <t>"이번 Journey 진행상태" — 9단계 순서·상태 pill</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
@@ -3302,44 +3302,44 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>/journey/fork(SCR009)로 이동</t>
+          <t>실데이터 렌더링</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /journeys/{id}</t>
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[코드-스펙 괴리] 이 API 응답엔 레포·이슈 정보(meta)가 없어, 새로고침 시 이 카드 자체는 복구되지만 이후 화면(SCR009~013)은 meta 없이는 정상 동작하지 않는다 — '새로고침 복구용'이라는 이름이 이 카드에만 해당됨</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>SCR009</t>
+          <t>SCR008</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Fork·Clone 통합</t>
+          <t>Journey 개요</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>SCR009-1</t>
+          <t>SCR008-3</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>카드</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>h1 "Fork &amp; Clone · 내 작업 공간 준비하기"</t>
+          <t>"단계별 스킵·자동화 Matrix" — 부록B 정적 표 + 단계별 "다음부터 기본 건너뛰기" 토글(실제 스킵 버튼이 있는 4단계 FORK·CLONE/REPO_ISSUE_BRIEF/QUESTION_COACH/COMMIT_PUSH·PR만 노출 — 매트릭스 문구와 실제 UI 불일치 방지)</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
@@ -3349,44 +3349,44 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>토글 변경 시 PATCH /journeys/step-preferences(API-20) upsert</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /journeys/{id}, PATCH /journeys/step-preferences</t>
         </is>
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] 이전 판은 표19 설정 변경 UI 요구를 진단만 하고 '보기전용'이었음 — 토글 UI를 실제 요구로 승격(요구사항정의서 REQ-014 참고)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>SCR009</t>
+          <t>SCR008</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Fork·Clone 통합</t>
+          <t>Journey 개요</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>SCR009-2</t>
+          <t>SCR008-4</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>표</t>
+          <t>버튼(Link)</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>개념설명(Fork=계정복사 / Clone=컴퓨터내려받기)</t>
+          <t>"Fork부터 시작할게요 →"</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>/journey/fork(SCR009)로 이동</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -3423,17 +3423,17 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>SCR009-3</t>
+          <t>SCR009-1</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>"⚡ 이 단계 자동화하기"</t>
+          <t>h1 "Fork &amp; Clone · 내 작업 공간 준비하기"</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
@@ -3443,17 +3443,17 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>disabled=busy 또는 meta없음</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>POST /automations/fork</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>[코드-스펙 괴리] 실제 GitHub API 미호출(시뮬레이션)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -3470,27 +3470,27 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>SCR009-4</t>
+          <t>SCR009-2</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>콜아웃(조건부)</t>
+          <t>표</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>자동화 성공 결과 안내(forkedRepoUrl)</t>
+          <t>개념설명(Fork=계정복사 / Clone=컴퓨터내려받기)</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>autoState==='success'일 때</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>SCR009-5</t>
+          <t>SCR009-3</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -3527,27 +3527,27 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>"자동화 실패 시나리오 보기"(데모)</t>
+          <t>"⚡ 이 단계 자동화하기"</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>클라이언트 상태만 토글</t>
+          <t>disabled=busy 또는 meta없음, 첫 클릭 시 동의 모달 표시</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POST /automations/fork</t>
         </is>
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] 실제 GitHub API로 Fork 생성(기존 Fork 있으면 재사용)하도록 요구 승격 — 이전 판 '시뮬레이션'은 진단만 있었음</t>
         </is>
       </c>
     </row>
@@ -3564,17 +3564,17 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>SCR009-6</t>
+          <t>SCR009-4</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>콜아웃(조건부)</t>
+          <t>모달(조건부)</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>실패 안내 + 수동 Fork 링크</t>
+          <t>동의 모달 — "Fork 자동화에 동의합니다" + 대상 저장소 fullName 표시 + 확인 버튼</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
@@ -3584,17 +3584,17 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>autoState==='failed'일 때</t>
+          <t>FORK_AUTOMATION Consent 미보유 사용자가 위 버튼 첫 클릭 시(이미 동의했으면 대상 확인 문구만 표시, 모달 생략)</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POST /consents</t>
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>BR07. [코드-스펙 괴리][중대] '저장소 링크 바로 열기' href가 실제로는 해당 레포가 아니라 하드코딩된 'https://github.com'(홈)이다 — BR07의 핵심인 수동 Fallback이 사용자를 막다른 곳에 내려놓는다. repo.repoUrl로 교체 필요(1줄 수정)</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] BR05·BR06이 요구하는 '자동화 동의 확인'이 실행 경로에 전혀 없던 것을 신규 UI로 승격(요구사항정의서 REQ-015 참고)</t>
         </is>
       </c>
     </row>
@@ -3611,32 +3611,32 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>SCR009-7</t>
+          <t>SCR009-5</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>코드블록</t>
+          <t>콜아웃(조건부)</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>git clone 명령</t>
+          <t>자동화 성공 결과 안내(forkedRepoUrl)</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>postAutomationClonePrepare() 진입 시 자동 조회</t>
+          <t>autoState==='success'일 때</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>POST /automations/clone/prepare</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I64" s="7" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>SCR009-8</t>
+          <t>SCR009-6</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -3668,17 +3668,17 @@
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>"📋 git 명령 복사"</t>
+          <t>"자동화 실패 시나리오 보기"(데모)</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>disabled=명령 없음, navigator.clipboard.writeText</t>
+          <t>클라이언트 상태만 토글</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -3705,37 +3705,37 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>SCR009-9</t>
+          <t>SCR009-7</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>콜아웃(조건부)</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>"💻 IDE에서 열기"</t>
+          <t>실패 안내 + 수동 Fork 링크</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>deepLinkUrl로 이동 시도</t>
+          <t>autoState==='failed'일 때</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>POST /ide-launch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>[코드-스펙 괴리] ide 파라미터 'VSCODE' 하드코딩</t>
+          <t>BR07. [코드-스펙 괴리][중대] '저장소 링크 바로 열기' href가 실제로는 해당 레포가 아니라 하드코딩된 'https://github.com'(홈)이다 — BR07의 핵심인 수동 Fallback이 사용자를 막다른 곳에 내려놓는다. repo.repoUrl로 교체 필요(1줄 수정)</t>
         </is>
       </c>
     </row>
@@ -3752,32 +3752,32 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>SCR009-10</t>
+          <t>SCR009-8</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>콜아웃(조건부)</t>
+          <t>코드블록</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>IDE 실행 결과 안내</t>
+          <t>git clone 명령</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>ideOpened===true일 때</t>
+          <t>postAutomationClonePrepare() 진입 시 자동 조회</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POST /automations/clone/prepare</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -3799,17 +3799,17 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>SCR009-11</t>
+          <t>SCR009-9</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>수동 Fallback 안내 note</t>
+          <t>"📋 git 명령 복사"</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>상시 노출</t>
+          <t>disabled=명령 없음, navigator.clipboard.writeText</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
-          <t>BR07</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>SCR009-12</t>
+          <t>SCR009-10</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>"이 단계 건너뛰기(다음부터 숨김)"</t>
+          <t>"💻 IDE에서 열기"</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -3866,17 +3866,17 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>FORK·CLONE 두 단계 SKIP 순차 PATCH</t>
+          <t>deepLinkUrl로 이동 시도(ide=REQ-005 저장 primaryIde)</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>PATCH /journeys/{id}/steps/FORK, PATCH .../CLONE</t>
+          <t>POST /ide-launch</t>
         </is>
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>화면 통합으로 개별 스킵 불가. [코드-스펙 괴리][중대] '(다음부터 숨김)'은 거짓 약속이다 — StepPreference 테이블(데이터사전 ENT-25)이 미사용이라 스킵 선택이 어디에도 저장되지 않고, 다음 Journey에서도 이 화면이 그대로 다시 나온다. [설계제안] MVP 문구에서 '(다음부터 숨김)' 삭제</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] ide 파라미터 'VSCODE' 하드코딩을 진단만 하던 것에서 primaryIde 사용을 요구로 승격</t>
         </is>
       </c>
     </row>
@@ -3893,54 +3893,54 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>SCR009-13</t>
+          <t>SCR009-11</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>콜아웃(조건부)</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>"Fork·Clone 확인했어요·다음 →"</t>
+          <t>IDE 실행 결과 안내</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>FORK·CLONE 두 단계 COMPLETE 순차 PATCH 후 /journey/brief(SCR010) 이동</t>
+          <t>ideOpened===true일 때</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>PATCH /journeys/{id}/steps/FORK, PATCH .../CLONE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>[v1.1 설계target] 부분실패 재시도(FORK_DONE 유지) 로직 미구현</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>SCR010</t>
+          <t>SCR009</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Repo·Issue Brief</t>
+          <t>Fork·Clone 통합</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>SCR010-1</t>
+          <t>SCR009-12</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>h1 "레포 &amp; 이슈, 쉽게 정리해줄게요"</t>
+          <t>수동 Fallback 안내 note</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>상시 노출</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -3970,34 +3970,34 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR07</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>SCR010</t>
+          <t>SCR009</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Repo·Issue Brief</t>
+          <t>Fork·Clone 통합</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>SCR010-2</t>
+          <t>SCR009-13</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>레포 설명 · 언어 태그 · 격려 문구</t>
+          <t>"이 단계 건너뛰기(다음부터 숨김)"</t>
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr">
@@ -4007,44 +4007,44 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>실데이터</t>
+          <t>FORK·CLONE 두 단계 SKIP 순차 PATCH + StepPreference(FORK/CLONE, defaultSkip=true) upsert</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>GET /recommendations/repositories</t>
+          <t>PATCH /journeys/{id}/steps/FORK, PATCH .../CLONE, PATCH /journeys/step-preferences(API-20)</t>
         </is>
       </c>
       <c r="I72" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>화면 통합으로 개별 스킵 불가. [정정 2026-07-20, 요구사항으로 승격] '(다음부터 숨김)' 문구가 StepPreference 미사용으로 거짓 약속이었던 것을 실제 저장·적용 요구로 승격(문구 삭제안은 폐기 — 요구사항정의서 REQ-018 참고)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>SCR010</t>
+          <t>SCR009</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Repo·Issue Brief</t>
+          <t>Fork·Clone 통합</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>SCR010-3</t>
+          <t>SCR009-14</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>이슈 제목 · 요약 · 표(현재문제/기대결과/완료기준) · 난이도/범위</t>
+          <t>"Fork·Clone 확인했어요·다음 →"</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
@@ -4054,17 +4054,17 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>실데이터</t>
+          <t>FORK·CLONE 두 단계 COMPLETE 순차 PATCH 후 /journey/brief(SCR010) 이동</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>GET /repositories/{id}/issues</t>
+          <t>PATCH /journeys/{id}/steps/FORK, PATCH .../CLONE</t>
         </is>
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[v1.1 설계target] 부분실패 재시도(FORK_DONE 유지) 로직 미구현</t>
         </is>
       </c>
     </row>
@@ -4081,27 +4081,27 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>SCR010-4</t>
+          <t>SCR010-1</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>"📖 배경 지식" — 쉬운 설명 1~2문장 + 수정 전 원본 코드 미리보기</t>
+          <t>h1 "레포 &amp; 이슈, 쉽게 정리해줄게요"</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>coachData 정적 콘텐츠, TITLE_TO_KEY 매칭(실패 시 typo 폴백)</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>[v1.1 설계target] BR08 예외 허용 범위, 사전정의 7개 이슈에만 정확 매칭</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -4128,17 +4128,17 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>SCR010-5</t>
+          <t>SCR010-2</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>카드</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>"학습하며 수정하기 →"</t>
+          <t>레포 설명 · 언어 태그 · 격려 문구</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
@@ -4148,12 +4148,12 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>/journey/coach(SCR011)로 이동</t>
+          <t>실데이터</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>PATCH /journeys/{id}/steps/REPO_ISSUE_BRIEF</t>
+          <t>GET /recommendations/repositories</t>
         </is>
       </c>
       <c r="I75" s="7" t="inlineStr">
@@ -4165,27 +4165,27 @@
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>SCR011</t>
+          <t>SCR010</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>질문 Coach</t>
+          <t>Repo·Issue Brief</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>SCR011-1</t>
+          <t>SCR010-3</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>카드</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>h1 "학습하며 수정하기"</t>
+          <t>이슈 제목 · 요약 · 표(현재문제/기대결과/완료기준) · 난이도/범위</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
@@ -4195,12 +4195,12 @@
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>정적(phase별 리드문구 변경)</t>
+          <t>실데이터</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /repositories/{id}/issues</t>
         </is>
       </c>
       <c r="I76" s="7" t="inlineStr">
@@ -4212,27 +4212,27 @@
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>SCR011</t>
+          <t>SCR010</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>질문 Coach</t>
+          <t>Repo·Issue Brief</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>SCR011-2</t>
+          <t>SCR010-4</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>stepper</t>
+          <t>링크</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>탐색 단계 표시(① 검색어 고르기 ② 결과에서 파일 찾기)</t>
+          <t>"이슈 원문 보기 ↗"</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>es state 기준</t>
+          <t>issue.url, 새 탭으로 열기</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
@@ -4252,44 +4252,44 @@
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] 부록B '원문 링크 항상 제공' 제약이 완전누락이었던 것을 승격(요구사항정의서 REQ-019 참고)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>SCR011</t>
+          <t>SCR010</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>질문 Coach</t>
+          <t>Repo·Issue Brief</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>SCR011-3</t>
+          <t>SCR010-5</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(3, 순차)</t>
+          <t>카드</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>검색어 선택지 → grep 결과 선택지</t>
+          <t>"📖 배경 지식" — 쉬운 설명 1~2문장 + 수정 전 원본 코드 미리보기</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>클릭 전 정답 스타일 미노출(BR08), 정답/오답 각각 피드백</t>
+          <t>coachData 정적 콘텐츠, TITLE_TO_KEY 매칭(실패 시 typo 폴백)</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
@@ -4299,24 +4299,24 @@
       </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>BR08</t>
+          <t>[v1.1 설계target] BR08 예외 허용 범위, 사전정의 7개 이슈에만 정확 매칭</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>SCR011</t>
+          <t>SCR010</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>질문 Coach</t>
+          <t>Repo·Issue Brief</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>SCR011-4</t>
+          <t>SCR010-6</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -4326,54 +4326,54 @@
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>"🤔 잘 모르겠어요"(힌트)</t>
+          <t>"이 단계 건너뛰기"</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>단계당 최대 3단계 힌트 순차 노출</t>
+          <t>PATCH .../REPO_ISSUE_BRIEF(action=SKIP) → /journey/coach 이동</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PATCH /journeys/{id}/steps/REPO_ISSUE_BRIEF</t>
         </is>
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] BR05·부록B 스킵 버튼 4곳 중 하나 — 이전 판엔 진단만 있었음(요구사항정의서 REQ-020 참고)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>SCR011</t>
+          <t>SCR010</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>질문 Coach</t>
+          <t>Repo·Issue Brief</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>SCR011-5</t>
+          <t>SCR010-7</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>카드목록</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>대안(approach) 비교 — 이름·난이도·트레이드오프·수정파일수</t>
+          <t>"학습하며 수정하기 →"</t>
         </is>
       </c>
       <c r="F80" s="7" t="inlineStr">
@@ -4383,12 +4383,12 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>coachData 정적</t>
+          <t>/journey/coach(SCR011)로 이동</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PATCH /journeys/{id}/steps/REPO_ISSUE_BRIEF</t>
         </is>
       </c>
       <c r="I80" s="7" t="inlineStr">
@@ -4410,17 +4410,17 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>SCR011-6</t>
+          <t>SCR011-1</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>코드블록</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>블록 선택(어디를 고칠까)</t>
+          <t>h1 "학습하며 수정하기"</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>클릭 시 정답/오답 피드백</t>
+          <t>정적(phase별 리드문구 변경)</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>BR08</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -4457,17 +4457,17 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>SCR011-7</t>
+          <t>SCR011-2</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>버튼그룹(3지선다)</t>
+          <t>stepper</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>객관식 질문 + '왜 그렇게 판단했나요' 후속질문</t>
+          <t>탐색 단계 표시(① 검색어 고르기 ② 결과에서 파일 찾기)</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>정답 선택 시에만 후속질문 노출</t>
+          <t>es state 기준</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>BR09</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -4504,27 +4504,27 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>SCR011-8</t>
+          <t>SCR011-3</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>사고흔적 램프(4종)</t>
+          <t>버튼그룹(3, 순차)</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>독립사고 · 추측사실구분 · 근거인용 · 질문습관</t>
+          <t>검색어 선택지 → grep 결과 선택지</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>조건 충족 시 점등</t>
+          <t>클릭 전 정답 스타일 미노출(BR08), 정답/오답 각각 피드백</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR08</t>
         </is>
       </c>
     </row>
@@ -4551,17 +4551,17 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>SCR011-9</t>
+          <t>SCR011-4</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>입력필드</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>자유 질문 입력 + '질문' 버튼</t>
+          <t>"🤔 잘 모르겠어요"(힌트)</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>2자 미만 시 경고, 제출 시 칭찬 문구 순환 노출</t>
+          <t>단계당 최대 3단계 힌트 순차 노출</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
@@ -4598,17 +4598,17 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>SCR011-10</t>
+          <t>SCR011-5</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>카드목록</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>"다음 →" / "코치 마치고 커밋·PR로 →"</t>
+          <t>대안(approach) 비교 — 이름·난이도·트레이드오프·수정파일수</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
@@ -4618,44 +4618,44 @@
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>마지막 단계에서 /journey/ship(SCR012)로 이동</t>
+          <t>coachData 정적</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>PATCH /journeys/{id}/steps/QUESTION_COACH</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>[v1.1 설계target] 답변·힌트 이력 서버 미저장(learning 도메인 dormant)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>SCR012-1</t>
+          <t>SCR011-6</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>코드블록</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>h1 "이제 커밋하고 PR로 반영 요청해요"</t>
+          <t>블록 선택(어디를 고칠까)</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>클릭 시 정답/오답 피드백</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
@@ -4675,34 +4675,34 @@
       </c>
       <c r="I86" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR08</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>SCR012-2</t>
+          <t>SCR011-7</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>표</t>
+          <t>버튼그룹(3지선다)</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>개념설명(커밋/Push/PR 정의)</t>
+          <t>객관식 질문 + '왜 그렇게 판단했나요' 후속질문</t>
         </is>
       </c>
       <c r="F87" s="7" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>정답 선택 시에만 후속질문 노출</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
@@ -4722,34 +4722,34 @@
       </c>
       <c r="I87" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR09</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>SCR012-3</t>
+          <t>SCR011-8</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>코드블록</t>
+          <t>버튼그룹(검증 단계)</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>커밋 명령 3줄(checkout -b / commit -am / push)</t>
+          <t>마지막 단계 '검증' 질문 — '수정이 맞다는 걸 어떻게 검증할까요' 유형(테스트 통과 포함 선택지)</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>정적, 각 줄 설명 포함</t>
+          <t>coachData 정적, 각 시나리오 마지막에 항상 존재</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
@@ -4769,34 +4769,34 @@
       </c>
       <c r="I88" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[확인완료 2026-07-20] UC05 검증 관점 질문은 coachData.ts에 이미 존재함을 확인 — 신규 요구 아님</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>SCR012-4</t>
+          <t>SCR011-9</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>사고흔적 램프(4종)</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>좋은/나쁜 커밋 메시지 예시</t>
+          <t>독립사고 · 추측사실구분 · 근거인용 · 질문습관</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>정적</t>
+          <t>조건 충족 시 점등</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
@@ -4823,37 +4823,37 @@
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>SCR012-5</t>
+          <t>SCR011-10</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>입력필드</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>PR 템플릿(What/Why/How tested/Fixes)</t>
+          <t>자유 질문 입력 + '질문' 버튼</t>
         </is>
       </c>
       <c r="F90" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>정적, 각 필드 설명 포함</t>
+          <t>2자 미만 시 경고, 제출 시 칭찬 문구 순환 노출</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
@@ -4870,27 +4870,27 @@
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>SCR012-6</t>
+          <t>SCR011-11</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>입력필드</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>"💻 바로 실습하기(IDE 열기) ↗"</t>
+          <t>기여 계획 한 줄 입력 — placeholder "이 이슈를 어떻게 해결할지 한 문장으로 적어보세요"</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>로컬 state만 토글</t>
+          <t>ContributionPlan.summary로 저장(스킵 시 생략)</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
@@ -4910,101 +4910,101 @@
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
-          <t>[코드-스펙 괴리] postIdeLaunch() 미호출, 실제 실행 아님</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] UC05 기여 계획 작성 UI 완전누락을 신설(요구사항정의서 REQ-024 참고)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>SCR012-7</t>
+          <t>SCR011-12</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>체크리스트(3항목, 토글)</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>코드 수정했다 / 커밋·push 했다 / PR을 열었다</t>
+          <t>"이 단계 건너뛰기"</t>
         </is>
       </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>로컬 state만, 제출 차단 안 함</t>
+          <t>PATCH .../QUESTION_COACH(action=SKIP) → /journey/ship 이동(기여 계획 입력 생략)</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PATCH /journeys/{id}/steps/QUESTION_COACH</t>
         </is>
       </c>
       <c r="I92" s="7" t="inlineStr">
         <is>
-          <t>[v1.1 설계target] 서버 저장(GitOperationCheckpoint) 미구현</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] BR05·부록B 스킵 버튼 4곳 중 하나(요구사항정의서 REQ-024 참고)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>SCR012</t>
+          <t>SCR011</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Commit·PR</t>
+          <t>질문 Coach</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>SCR012-8</t>
+          <t>SCR011-13</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>콜아웃</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>응답시간 기대 안내(메인테이너 첫 반응 예상 약 N시간)</t>
+          <t>"다음 →" / "코치 마치고 커밋·PR로 →"</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>avgFeedbackHours 있을 때만 노출</t>
+          <t>마지막 단계에서 /journey/ship(SCR012)로 이동</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>GET /recommendations/repositories</t>
+          <t>PATCH /journeys/{id}/steps/QUESTION_COACH</t>
         </is>
       </c>
       <c r="I93" s="7" t="inlineStr">
         <is>
-          <t>BR09</t>
+          <t>[v1.1 설계target] 답변·힌트 이력 서버 미저장(learning 도메인 dormant)</t>
         </is>
       </c>
     </row>
@@ -5021,17 +5021,17 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>SCR012-9</t>
+          <t>SCR012-1</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>입력필드</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>PR URL</t>
+          <t>h1 "이제 커밋하고 PR로 반영 요청해요"</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>placeholder 예시 표시</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
@@ -5068,27 +5068,27 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>SCR012-10</t>
+          <t>SCR012-2</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>텍스트(조건부)</t>
+          <t>표</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>에러: URL 형식 오류 / 등록 실패</t>
+          <t>개념설명(커밋/Push/PR 정의)</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>정규식 검증 실패 시</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
-          <t>[설계제안] 형식 안내 문구 명문화</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5115,17 +5115,17 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>SCR012-11</t>
+          <t>SCR012-3</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>코드블록</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>"PR 등록완료·상태확인하러가기 →" / "등록중…"</t>
+          <t>커밋 명령 3줄(checkout -b / commit -am / push)</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
@@ -5135,12 +5135,12 @@
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>disabled=진행중 또는 URL없음, 성공 시 /journey/monitoring(SCR013) 이동</t>
+          <t>정적, 각 줄 설명 포함</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
         <is>
-          <t>POST /pull-requests, GET /pull-requests/{id}/status, PATCH .../COMMIT_PUSH, PATCH .../PR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I96" s="7" t="inlineStr">
@@ -5152,17 +5152,17 @@
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>SCR013-1</t>
+          <t>SCR012-4</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -5172,12 +5172,12 @@
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>h1 "PR Monitoring"</t>
+          <t>좋은/나쁜 커밋 메시지 예시</t>
         </is>
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
@@ -5199,37 +5199,37 @@
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>SCR013-2</t>
+          <t>SCR012-5</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>상태분기</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>연결된 PR 없음</t>
+          <t>PR 템플릿(What/Why/How tested/Fixes)</t>
         </is>
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>pullRequest===null일 때 안내만 표시</t>
+          <t>정적, 각 필드 설명 포함</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
@@ -5246,84 +5246,84 @@
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>SCR013-3</t>
+          <t>SCR012-6</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>배지</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>MERGED / CLOSED_UNMERGED / OPEN / UNKNOWN</t>
+          <t>"💻 바로 실습하기(IDE 열기) ↗"</t>
         </is>
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>STATE_COPY 매핑 렌더</t>
+          <t>postIdeLaunch(ide=primaryIde) 호출 → deepLinkUrl로 이동, 실패 시 수동 안내</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POST /ide-launch</t>
         </is>
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
-          <t>BR11</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] postIdeLaunch() 미호출을 진단만 하던 것에서 REQ-017과 동일한 실제 호출로 요구 승격(요구사항정의서 REQ-025 참고)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>SCR013-4</t>
+          <t>SCR012-7</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>체크리스트(3항목, 토글)</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>조회 시각 · 출처</t>
+          <t>코드 수정했다 / 커밋·push 했다 / PR을 열었다</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>실데이터</t>
+          <t>로컬 state만, 제출 차단 안 함</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr">
@@ -5333,138 +5333,138 @@
       </c>
       <c r="I100" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>[v1.1 설계target] 서버 저장(GitOperationCheckpoint) 미구현</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>SCR013-5</t>
+          <t>SCR012-8</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>링크</t>
+          <t>콜아웃</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>"GitHub에서 PR 원문 보기 ↗"</t>
+          <t>응답시간 기대 안내(메인테이너 첫 반응 예상 약 N시간)</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>새 탭</t>
+          <t>avgFeedbackHours 있을 때만 노출</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /recommendations/repositories</t>
         </is>
       </c>
       <c r="I101" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR09</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>SCR013-6</t>
+          <t>SCR012-9</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>카드(조건부)</t>
+          <t>링크</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>"⏳ 기다리는 동안" — 경과시간 vs 메인테이너 첫반응 예상시간</t>
+          <t>"GitHub에서 PR 열러 가기 ↗"</t>
         </is>
       </c>
       <c r="F102" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>state==='OPEN' &amp;&amp; avgFeedbackHours 있을 때만</t>
+          <t>fork된 저장소 compare 페이지(https://github.com/{owner}/{repo}/compare)</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr">
         <is>
-          <t>GET /recommendations/repositories</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I102" s="7" t="inlineStr">
         <is>
-          <t>BR09. [코드-스펙 괴리][중대] 경과시간 기준 시각이 '그린커밋에 PR을 등록한 시각'이지 'GitHub에서 PR을 연 시각'이 아니다 — 예전에 연 PR을 지금 등록하면 '0시간째'로 잘못 표시된다. 게다가 상태 자체는 등록 시점 1회 조회로 고정돼 있어 시간만 흐르고 상태는 갱신되지 않는다(재조회 버튼 없음) — 감시하는 것처럼 보이지만 실제로는 아무것도 감시하지 않는 구조</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] F015 '페이지 연결' 요구 완전누락을 신설(요구사항정의서 REQ-027 참고)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>SCR013-7</t>
+          <t>SCR012-10</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>카드</t>
+          <t>입력필드</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>"이 화면이 나중에 보여줄 것"(F017 확장 예고)</t>
+          <t>PR URL</t>
         </is>
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>정적, 미구현 항목 정직 안내</t>
+          <t>placeholder 예시 표시</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr">
@@ -5481,74 +5481,74 @@
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>SCR013</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>PR Monitoring</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>SCR013-8</t>
+          <t>SCR012-11</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>버튼</t>
+          <t>텍스트(조건부)</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>"결과 화면 보기 →"</t>
+          <t>에러: URL 형식 오류 / 등록 실패</t>
         </is>
       </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>/journey/result(SCR014)로 이동</t>
+          <t>정규식 검증 실패 시</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
         <is>
-          <t>PATCH /journeys/{id}/steps/MONITORING</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I104" s="7" t="inlineStr">
         <is>
-          <t>[코드-스펙 괴리][중대] 상태 재조회 버튼이 이 화면에 없다 — 정상 흐름에서 방금 등록한 PR은 거의 항상 OPEN이라, SCR014의 MERGED/CLOSED 결과화면은 실질적으로 도달 불가능하다. [설계제안] 기존 GET /pull-requests/{id}/status를 재호출하는 '지금 다시 확인하기' 버튼 추가</t>
+          <t>[설계제안] 형식 안내 문구 명문화</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>SCR014</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>결과</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>SCR014-1</t>
+          <t>SCR012-12</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>상태분기</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>MERGED / CLOSED_UNMERGED / OPEN / UNKNOWN / (PR미등록 시 데모모드)</t>
+          <t>"PR 등록완료·상태확인하러가기 →" / "등록중…"</t>
         </is>
       </c>
       <c r="F105" s="7" t="inlineStr">
@@ -5558,101 +5558,101 @@
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>pullRequest.status.state 기준 4+1분기</t>
+          <t>disabled=진행중 또는 URL없음, 성공 시 /journey/monitoring(SCR013) 이동</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POST /pull-requests, GET /pull-requests/{id}/status, PATCH .../COMMIT_PUSH, PATCH .../PR</t>
         </is>
       </c>
       <c r="I105" s="7" t="inlineStr">
         <is>
-          <t>BR11</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>SCR014</t>
+          <t>SCR012</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>결과</t>
+          <t>Commit·PR</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>SCR014-2</t>
+          <t>SCR012-13</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>[MERGED뷰] 텍스트+카드</t>
+          <t>버튼</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>"축하해요, 머지됐어요! 🎉" + 역량미터 2종(정적) + 버튼2개("더 깊은 미션 "도전 →"/"나의 기여 기록 보기")</t>
+          <t>"이 단계 건너뛰기" — "PR 미등록 상태로 마칠게요" 확인 문구</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
-          <t>state==='MERGED'</t>
+          <t>PATCH .../COMMIT_PUSH·PATCH .../PR(둘 다 action=SKIP) → PullRequestLink 생성하지 않고 MONITORING·RESULT(PR상태 4분기)를 건너뛴 채 Journey를 SKIPPED_NO_PR로 종료 → /recommend/repositories(다음 미션)로 직행</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PATCH /journeys/{id}/steps/COMMIT_PUSH, PATCH /journeys/{id}/steps/PR</t>
         </is>
       </c>
       <c r="I106" s="7" t="inlineStr">
         <is>
-          <t>역량미터는 [범위밖](F023). [코드-스펙 괴리] 등록 직후 1회 조회 구조상(SCR013-6 참고) 정상 흐름에서 이 뷰 자체에 도달하기 어렵다. [코드-스펙 괴리] '더 깊은 미션 도전 →'이 실제로는 REQ-031의 '비슷한 다른 이슈 찾기'와 똑같이 /recommend/repositories로 간다(추천은 '깊이'를 반영 안 하는 정적 시드 6개) — 랜딩페이지(SCR001-6/7)와 같은 유형의 텍스트만 다른 중복 버튼</t>
+          <t>[정정 2026-07-20, 요구사항으로 승격] BR05(모든 단계 스킵 가능)와 BR10(사용자가 연결한 PR만 수집)이 충돌해 보이지 않도록 'PR 미등록으로 Journey 종료'를 명확한 흐름으로 신설(요구사항정의서 REQ-027 참고)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t>SCR014</t>
+          <t>SCR013</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>결과</t>
+          <t>PR Monitoring</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>SCR014-3</t>
+          <t>SCR013-1</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>[CLOSED뷰] 텍스트+배지</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>"이번엔 머지되지 않았어요" + Closed사유 pill 5종(참고용) + 버튼2개("보완해서 다시 요청 →"/"비슷한 다른 이슈 찾기")</t>
+          <t>h1 "PR Monitoring"</t>
         </is>
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>state==='CLOSED_UNMERGED', reason은 항상 'Unknown'</t>
+          <t>정적</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
@@ -5662,34 +5662,34 @@
       </c>
       <c r="I107" s="7" t="inlineStr">
         <is>
-          <t>BR11, BR14. [코드-스펙 괴리][중대] '보완해서 다시 요청하기 →'의 실제 목적지가 /journey/coach(SCR011)다 — Coach는 7개 이슈용 정적 퀴즈라 다시 가도 같은 문제만 나오고, PR을 다시 등록하려면 SCR012로 가야 한다. 게다가 이 Journey의 QUESTION_COACH·COMMIT_PUSH·PR 단계는 이미 COMPLETED이고 재오픈 로직이 없어 흐름상 성립하지 않는 목적지다. [설계제안] 목적지를 SCR012로 변경</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>SCR014</t>
+          <t>SCR013</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>결과</t>
+          <t>PR Monitoring</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>SCR014-4</t>
+          <t>SCR013-2</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>[OPEN뷰] 텍스트+링크</t>
+          <t>상태분기</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>"PR이 아직 열려 있어요" + BR14 안내 + GitHub링크 + 버튼</t>
+          <t>연결된 PR 없음</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>state==='OPEN'</t>
+          <t>pullRequest===null일 때 안내만 표시</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr">
@@ -5709,44 +5709,44 @@
       </c>
       <c r="I108" s="7" t="inlineStr">
         <is>
-          <t>BR14</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t>SCR014</t>
+          <t>SCR013</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>결과</t>
+          <t>PR Monitoring</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>SCR014-5</t>
+          <t>SCR013-3</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>[UNKNOWN뷰] 텍스트+링크</t>
+          <t>배지</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>"상태를 확인하지 못했어요" + GitHub링크</t>
+          <t>MERGED / CLOSED_UNMERGED / OPEN / UNKNOWN</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>그 외 모든 경우</t>
+          <t>STATE_COPY 매핑 렌더</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr">
@@ -5756,24 +5756,24 @@
       </c>
       <c r="I109" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR11</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>SCR015</t>
+          <t>SCR013</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>알림</t>
+          <t>PR Monitoring</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>SCR015-1</t>
+          <t>SCR013-4</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -5783,54 +5783,54 @@
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>"알림 보관함 🔔" + mock 3건</t>
+          <t>조회 시각 · 출처</t>
         </is>
       </c>
       <c r="F110" s="7" t="inlineStr">
         <is>
-          <t>조건부(현재 항상 표시)</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
         <is>
-          <t>MOCK_NOTIFICATIONS 하드코딩, API 호출 안 함</t>
+          <t>실데이터</t>
         </is>
       </c>
       <c r="H110" s="7" t="inlineStr">
         <is>
-          <t>GET /notifications(호출 안 함)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I110" s="7" t="inlineStr">
         <is>
-          <t>[범위밖][코드-스펙 괴리] 실데이터처럼 보이는 mock — 우선순위 1위 리스크</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t>SCR016</t>
+          <t>SCR013</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>나의 기여</t>
+          <t>PR Monitoring</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>SCR016-1</t>
+          <t>SCR013-5</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>섹션</t>
+          <t>링크</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>"기여 History"(실데이터)</t>
+          <t>"GitHub에서 PR 원문 보기 ↗"</t>
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>실제 조회</t>
+          <t>새 탭</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr">
         <is>
-          <t>GET /history</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I111" s="7" t="inlineStr">
@@ -5857,92 +5857,562 @@
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>SCR016</t>
+          <t>SCR013</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>나의 기여</t>
+          <t>PR Monitoring</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>SCR016-2</t>
+          <t>SCR013-6</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>섹션</t>
+          <t>카드(조건부)</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>배지 · 사고역량지도 · 다음미션(정적)</t>
+          <t>"⏳ 기다리는 동안" — 경과시간 vs 메인테이너 첫반응 예상시간</t>
         </is>
       </c>
       <c r="F112" s="7" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>정적 상수, 실데이터 아님</t>
+          <t>state==='OPEN' &amp;&amp; avgFeedbackHours 있을 때만</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GET /recommendations/repositories</t>
         </is>
       </c>
       <c r="I112" s="7" t="inlineStr">
         <is>
-          <t>[범위밖](F023) — 실데이터 History와 같은 화면에 섞여 있어 혼동 주의</t>
+          <t>BR09. [코드-스펙 괴리][중대] 경과시간 기준 시각이 '그린커밋에 PR을 등록한 시각'이지 'GitHub에서 PR을 연 시각'이 아니다 — 예전에 연 PR을 지금 등록하면 '0시간째'로 잘못 표시된다. 게다가 상태 자체는 등록 시점 1회 조회로 고정돼 있어 시간만 흐르고 상태는 갱신되지 않는다(재조회 버튼 없음) — 감시하는 것처럼 보이지만 실제로는 아무것도 감시하지 않는 구조</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
         <is>
+          <t>SCR013</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>PR Monitoring</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>SCR013-7</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t>카드</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>"이 화면이 나중에 보여줄 것"(F017 확장 예고)</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="G113" s="7" t="inlineStr">
+        <is>
+          <t>정적, 미구현 항목 정직 안내</t>
+        </is>
+      </c>
+      <c r="H113" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I113" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>SCR013</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>PR Monitoring</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>SCR013-8</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>버튼</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>"결과 화면 보기 →"</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="G114" s="7" t="inlineStr">
+        <is>
+          <t>/journey/result(SCR014)로 이동</t>
+        </is>
+      </c>
+      <c r="H114" s="7" t="inlineStr">
+        <is>
+          <t>PATCH /journeys/{id}/steps/MONITORING</t>
+        </is>
+      </c>
+      <c r="I114" s="7" t="inlineStr">
+        <is>
+          <t>[코드-스펙 괴리][중대] 상태 재조회 버튼이 이 화면에 없다 — 정상 흐름에서 방금 등록한 PR은 거의 항상 OPEN이라, SCR014의 MERGED/CLOSED 결과화면은 실질적으로 도달 불가능하다. [설계제안] 기존 GET /pull-requests/{id}/status를 재호출하는 '지금 다시 확인하기' 버튼 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>SCR014</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>SCR014-1</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>상태분기</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>MERGED / CLOSED_UNMERGED / OPEN / UNKNOWN / (PR미등록 시 데모모드)</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>pullRequest.status.state 기준 4+1분기</t>
+        </is>
+      </c>
+      <c r="H115" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I115" s="7" t="inlineStr">
+        <is>
+          <t>BR11</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>SCR014</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>SCR014-2</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>[MERGED뷰] 텍스트+카드</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>"축하해요, 머지됐어요! 🎉" + 역량미터 2종(정적) + 버튼2개("더 깊은 미션 "도전 →"/"나의 기여 기록 보기")</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>조건부</t>
+        </is>
+      </c>
+      <c r="G116" s="7" t="inlineStr">
+        <is>
+          <t>state==='MERGED'</t>
+        </is>
+      </c>
+      <c r="H116" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I116" s="7" t="inlineStr">
+        <is>
+          <t>역량미터는 [범위밖](F023). [코드-스펙 괴리] 등록 직후 1회 조회 구조상(SCR013-6 참고) 정상 흐름에서 이 뷰 자체에 도달하기 어렵다. [코드-스펙 괴리] '더 깊은 미션 도전 →'이 실제로는 REQ-031의 '비슷한 다른 이슈 찾기'와 똑같이 /recommend/repositories로 간다(추천은 '깊이'를 반영 안 하는 정적 시드 6개) — 랜딩페이지(SCR001-6/7)와 같은 유형의 텍스트만 다른 중복 버튼</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>SCR014</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>SCR014-3</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>[CLOSED뷰] 텍스트+배지</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>"이번엔 머지되지 않았어요" + Closed사유 pill 5종(참고용) + 버튼2개("보완해서 다시 요청 →"/"비슷한 다른 이슈 찾기")</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>조건부</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>state==='CLOSED_UNMERGED', reason은 항상 'Unknown'</t>
+        </is>
+      </c>
+      <c r="H117" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I117" s="7" t="inlineStr">
+        <is>
+          <t>BR11, BR14. [코드-스펙 괴리][중대] '보완해서 다시 요청하기 →'의 실제 목적지가 /journey/coach(SCR011)다 — Coach는 7개 이슈용 정적 퀴즈라 다시 가도 같은 문제만 나오고, PR을 다시 등록하려면 SCR012로 가야 한다. 게다가 이 Journey의 QUESTION_COACH·COMMIT_PUSH·PR 단계는 이미 COMPLETED이고 재오픈 로직이 없어 흐름상 성립하지 않는 목적지다. [설계제안] 목적지를 SCR012로 변경</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>SCR014</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>SCR014-4</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t>[OPEN뷰] 텍스트+링크</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>"PR이 아직 열려 있어요" + BR14 안내 + GitHub링크 + 버튼</t>
+        </is>
+      </c>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>조건부</t>
+        </is>
+      </c>
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>state==='OPEN'</t>
+        </is>
+      </c>
+      <c r="H118" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I118" s="7" t="inlineStr">
+        <is>
+          <t>BR14</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t>SCR014</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>SCR014-5</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>[UNKNOWN뷰] 텍스트+링크</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>"상태를 확인하지 못했어요" + GitHub링크</t>
+        </is>
+      </c>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>조건부</t>
+        </is>
+      </c>
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>그 외 모든 경우</t>
+        </is>
+      </c>
+      <c r="H119" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I119" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>SCR015</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>알림</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>SCR015-1</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>텍스트</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>"알림 보관함 🔔" + mock 3건</t>
+        </is>
+      </c>
+      <c r="F120" s="7" t="inlineStr">
+        <is>
+          <t>조건부(현재 항상 표시)</t>
+        </is>
+      </c>
+      <c r="G120" s="7" t="inlineStr">
+        <is>
+          <t>MOCK_NOTIFICATIONS 하드코딩, API 호출 안 함</t>
+        </is>
+      </c>
+      <c r="H120" s="7" t="inlineStr">
+        <is>
+          <t>GET /notifications(호출 안 함)</t>
+        </is>
+      </c>
+      <c r="I120" s="7" t="inlineStr">
+        <is>
+          <t>[범위밖][코드-스펙 괴리] 실데이터처럼 보이는 mock — 우선순위 1위 리스크</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>SCR016</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>나의 기여</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>SCR016-1</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>섹션</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>"기여 History"(실데이터)</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>실제 조회</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr">
+        <is>
+          <t>GET /history</t>
+        </is>
+      </c>
+      <c r="I121" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t>SCR016</t>
+        </is>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>나의 기여</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>SCR016-2</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t>섹션</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>배지 · 사고역량지도 · 다음미션(정적)</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="inlineStr">
+        <is>
+          <t>정적 상수, 실데이터 아님</t>
+        </is>
+      </c>
+      <c r="H122" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I122" s="7" t="inlineStr">
+        <is>
+          <t>[범위밖](F023) — 실데이터 History와 같은 화면에 섞여 있어 혼동 주의</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
           <t>SCR017</t>
         </is>
       </c>
-      <c r="B113" s="7" t="inlineStr">
+      <c r="B123" s="7" t="inlineStr">
         <is>
           <t>설정</t>
         </is>
       </c>
-      <c r="C113" s="7" t="inlineStr">
+      <c r="C123" s="7" t="inlineStr">
         <is>
           <t>SCR017-1</t>
         </is>
       </c>
-      <c r="D113" s="7" t="inlineStr">
+      <c r="D123" s="7" t="inlineStr">
         <is>
           <t>텍스트</t>
         </is>
       </c>
-      <c r="E113" s="7" t="inlineStr">
+      <c r="E123" s="7" t="inlineStr">
         <is>
           <t>IDE·자동화·스킵·연동·삭제 UI 전부</t>
         </is>
       </c>
-      <c r="F113" s="7" t="inlineStr">
+      <c r="F123" s="7" t="inlineStr">
         <is>
           <t>조건부(장식용)</t>
         </is>
       </c>
-      <c r="G113" s="7" t="inlineStr">
+      <c r="G123" s="7" t="inlineStr">
         <is>
           <t>API 호출 0건, 모든 조작이 로컬 state 또는 무동작</t>
         </is>
       </c>
-      <c r="H113" s="7" t="inlineStr">
+      <c r="H123" s="7" t="inlineStr">
         <is>
           <t>없음</t>
         </is>
       </c>
-      <c r="I113" s="7" t="inlineStr">
+      <c r="I123" s="7" t="inlineStr">
         <is>
           <t>[범위밖] 백엔드 settings 컨트롤러 자체가 없음</t>
         </is>

</xml_diff>